<commit_message>
catching up on commits... July 2025
</commit_message>
<xml_diff>
--- a/annotation/Species_list_vs_CATAMI_2023_10.xlsx
+++ b/annotation/Species_list_vs_CATAMI_2023_10.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28129"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jjansen\Desktop\science\SouthernOceanBiodiversityMapping\ARC_Data\annotation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universitytasmania-my.sharepoint.com/personal/jan_jansen_utas_edu_au/Documents/science/SouthernOceanBiodiversityMapping/ARC_Data/annotation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EE14C21-F118-4AE1-8CE9-DB6576968DEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="68" documentId="13_ncr:1_{5EE14C21-F118-4AE1-8CE9-DB6576968DEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB103039-2FA5-4D94-B407-B08ED006A349}"/>
   <bookViews>
-    <workbookView xWindow="15030" yWindow="-18120" windowWidth="29040" windowHeight="18240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14415" yWindow="-16350" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="COVER_naming" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1611" uniqueCount="655">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1655" uniqueCount="660">
   <si>
     <t>Label</t>
   </si>
@@ -1986,6 +1986,21 @@
   </si>
   <si>
     <t>Biota - Matrix - UBS_B TemporaryLabelDoNotUse</t>
+  </si>
+  <si>
+    <t>AMC_Merge_With_2pc_500m</t>
+  </si>
+  <si>
+    <t>Biota - Cnidaria - Hydroids</t>
+  </si>
+  <si>
+    <t>Biota - Molluscs</t>
+  </si>
+  <si>
+    <t>Biota - Cnidaria - Corals - Black &amp; Octocorals - Branching (3D) - Non-fleshy - Bottle-brush</t>
+  </si>
+  <si>
+    <t>Biota - Sponges - Erect forms</t>
   </si>
 </sst>
 </file>
@@ -2080,7 +2095,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2126,13 +2141,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Bad" xfId="1" builtinId="27"/>
@@ -2224,6 +2236,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2513,36 +2529,37 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X138"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:Y138"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="54" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="70.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="76.44140625" customWidth="1"/>
-    <col min="6" max="6" width="68.44140625" style="11" customWidth="1"/>
-    <col min="7" max="7" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.109375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="48.7109375" customWidth="1"/>
+    <col min="5" max="5" width="60.5703125" customWidth="1"/>
+    <col min="6" max="6" width="68.42578125" style="11" customWidth="1"/>
+    <col min="7" max="7" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.140625" style="2" customWidth="1"/>
     <col min="10" max="10" width="9" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.33203125" style="5" customWidth="1"/>
-    <col min="14" max="14" width="17.33203125" customWidth="1"/>
-    <col min="15" max="15" width="5.6640625" style="5" customWidth="1"/>
-    <col min="16" max="16" width="50" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.21875" style="5" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="30.44140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="9.5546875" customWidth="1"/>
-    <col min="22" max="22" width="70.109375" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="17.109375" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="16" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5.28515625" style="5" customWidth="1"/>
+    <col min="14" max="14" width="26.7109375" customWidth="1"/>
+    <col min="15" max="15" width="3.5703125" style="5" customWidth="1"/>
+    <col min="16" max="16" width="12.140625" style="5" customWidth="1"/>
+    <col min="17" max="17" width="48.140625" customWidth="1"/>
+    <col min="18" max="18" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="30.42578125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.5703125" customWidth="1"/>
+    <col min="23" max="23" width="70.140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:25" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2589,34 +2606,37 @@
         <v>487</v>
       </c>
       <c r="P1" s="1" t="s">
+        <v>655</v>
+      </c>
+      <c r="Q1" s="1" t="s">
         <v>486</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>306</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>323</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>488</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>490</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>489</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -2648,17 +2668,17 @@
       <c r="L2">
         <v>5.0999999999999997E-2</v>
       </c>
-      <c r="Q2">
+      <c r="R2">
         <v>35</v>
       </c>
-      <c r="R2">
+      <c r="S2">
         <v>7.5999999999999998E-2</v>
       </c>
-      <c r="V2" s="2" t="s">
+      <c r="W2" s="2" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -2693,17 +2713,17 @@
       <c r="L3" s="4">
         <v>2E-3</v>
       </c>
-      <c r="Q3">
+      <c r="R3">
         <v>2</v>
       </c>
-      <c r="R3" s="4">
+      <c r="S3" s="4">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="V3" s="2" t="s">
+      <c r="W3" s="2" t="s">
         <v>448</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -2735,17 +2755,17 @@
       <c r="L4" s="4">
         <v>1.7999999999999999E-2</v>
       </c>
-      <c r="Q4">
+      <c r="R4">
         <v>16</v>
       </c>
-      <c r="R4">
+      <c r="S4">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="V4" s="2" t="s">
+      <c r="W4" s="2" t="s">
         <v>447</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -2773,17 +2793,17 @@
       <c r="L5">
         <v>0.126</v>
       </c>
-      <c r="Q5">
+      <c r="R5">
         <v>81</v>
       </c>
-      <c r="R5">
+      <c r="S5">
         <v>0.17599999999999999</v>
       </c>
-      <c r="V5" s="2" t="s">
+      <c r="W5" s="2" t="s">
         <v>446</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -2821,23 +2841,26 @@
       <c r="N6" t="s">
         <v>15</v>
       </c>
-      <c r="P6" t="s">
+      <c r="P6" s="11" t="s">
+        <v>566</v>
+      </c>
+      <c r="Q6" t="s">
         <v>15</v>
       </c>
-      <c r="Q6">
+      <c r="R6">
         <v>6</v>
       </c>
-      <c r="R6" s="4">
+      <c r="S6" s="4">
         <v>1.2999999999999999E-2</v>
       </c>
-      <c r="T6" t="s">
+      <c r="U6" t="s">
         <v>15</v>
       </c>
-      <c r="V6" s="2" t="s">
+      <c r="W6" s="2" t="s">
         <v>447</v>
       </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -2872,17 +2895,17 @@
       <c r="L7">
         <v>6.9000000000000006E-2</v>
       </c>
-      <c r="Q7">
+      <c r="R7">
         <v>45</v>
       </c>
-      <c r="R7">
+      <c r="S7">
         <v>9.8000000000000004E-2</v>
       </c>
-      <c r="V7" s="2" t="s">
+      <c r="W7" s="2" t="s">
         <v>484</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -2922,20 +2945,23 @@
       <c r="N8" t="s">
         <v>18</v>
       </c>
-      <c r="P8" t="s">
+      <c r="P8" s="11" t="s">
+        <v>569</v>
+      </c>
+      <c r="Q8" t="s">
         <v>18</v>
       </c>
-      <c r="Q8">
+      <c r="R8">
         <v>11</v>
       </c>
-      <c r="R8">
+      <c r="S8">
         <v>2.4E-2</v>
       </c>
-      <c r="V8" s="2" t="s">
+      <c r="W8" s="2" t="s">
         <v>484</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -2972,17 +2998,17 @@
       <c r="L9">
         <v>2.9000000000000001E-2</v>
       </c>
-      <c r="Q9">
+      <c r="R9">
         <v>18</v>
       </c>
-      <c r="R9">
+      <c r="S9">
         <v>3.9E-2</v>
       </c>
-      <c r="V9" s="2" t="s">
+      <c r="W9" s="2" t="s">
         <v>443</v>
       </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -3017,17 +3043,17 @@
       <c r="L10">
         <v>6.2E-2</v>
       </c>
-      <c r="Q10">
+      <c r="R10">
         <v>38</v>
       </c>
-      <c r="R10">
+      <c r="S10">
         <v>8.3000000000000004E-2</v>
       </c>
-      <c r="V10" s="2" t="s">
+      <c r="W10" s="2" t="s">
         <v>442</v>
       </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -3062,17 +3088,17 @@
       <c r="L11">
         <v>0.29099999999999998</v>
       </c>
-      <c r="Q11">
+      <c r="R11">
         <v>165</v>
       </c>
-      <c r="R11">
+      <c r="S11">
         <v>0.35899999999999999</v>
       </c>
-      <c r="V11" s="2" t="s">
+      <c r="W11" s="2" t="s">
         <v>441</v>
       </c>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -3107,17 +3133,17 @@
       <c r="L12">
         <v>9.6000000000000002E-2</v>
       </c>
-      <c r="Q12">
+      <c r="R12">
         <v>73</v>
       </c>
-      <c r="R12">
+      <c r="S12">
         <v>0.159</v>
       </c>
-      <c r="V12" s="2" t="s">
+      <c r="W12" s="2" t="s">
         <v>440</v>
       </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -3155,20 +3181,20 @@
       <c r="O13" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q13">
+      <c r="R13">
         <v>2</v>
       </c>
-      <c r="R13" s="4">
+      <c r="S13" s="4">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="S13" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V13" s="2" t="s">
+      <c r="T13" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W13" s="2" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>25</v>
       </c>
@@ -3205,17 +3231,17 @@
       <c r="L14">
         <v>0.23300000000000001</v>
       </c>
-      <c r="Q14">
+      <c r="R14">
         <v>148</v>
       </c>
-      <c r="R14">
+      <c r="S14">
         <v>0.32200000000000001</v>
       </c>
-      <c r="V14" s="2" t="s">
+      <c r="W14" s="2" t="s">
         <v>439</v>
       </c>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>26</v>
       </c>
@@ -3252,17 +3278,17 @@
       <c r="L15">
         <v>2.1999999999999999E-2</v>
       </c>
-      <c r="Q15">
+      <c r="R15">
         <v>19</v>
       </c>
-      <c r="R15">
+      <c r="S15">
         <v>4.1000000000000002E-2</v>
       </c>
-      <c r="V15" s="2" t="s">
+      <c r="W15" s="2" t="s">
         <v>438</v>
       </c>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>27</v>
       </c>
@@ -3299,17 +3325,17 @@
       <c r="L16">
         <v>0.224</v>
       </c>
-      <c r="Q16">
+      <c r="R16">
         <v>128</v>
       </c>
-      <c r="R16">
+      <c r="S16">
         <v>0.27900000000000003</v>
       </c>
-      <c r="V16" s="2" t="s">
+      <c r="W16" s="2" t="s">
         <v>437</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>28</v>
       </c>
@@ -3349,23 +3375,26 @@
       <c r="N17" t="s">
         <v>25</v>
       </c>
-      <c r="P17" t="s">
+      <c r="P17" s="11" t="s">
+        <v>586</v>
+      </c>
+      <c r="Q17" t="s">
         <v>25</v>
       </c>
-      <c r="Q17">
+      <c r="R17">
         <v>10</v>
       </c>
-      <c r="R17">
+      <c r="S17">
         <v>2.1999999999999999E-2</v>
       </c>
-      <c r="T17" t="s">
+      <c r="U17" t="s">
         <v>25</v>
       </c>
-      <c r="V17" s="2" t="s">
+      <c r="W17" s="2" t="s">
         <v>439</v>
       </c>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>29</v>
       </c>
@@ -3400,17 +3429,17 @@
       <c r="L18">
         <v>0.106</v>
       </c>
-      <c r="Q18">
+      <c r="R18">
         <v>70</v>
       </c>
-      <c r="R18">
+      <c r="S18">
         <v>0.153</v>
       </c>
-      <c r="V18" s="2" t="s">
+      <c r="W18" s="2" t="s">
         <v>435</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>30</v>
       </c>
@@ -3445,17 +3474,17 @@
       <c r="L19">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="Q19">
+      <c r="R19">
         <v>51</v>
       </c>
-      <c r="R19">
+      <c r="S19">
         <v>0.111</v>
       </c>
-      <c r="V19" s="2" t="s">
+      <c r="W19" s="2" t="s">
         <v>434</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>31</v>
       </c>
@@ -3490,17 +3519,17 @@
       <c r="L20">
         <v>0.15</v>
       </c>
-      <c r="Q20">
+      <c r="R20">
         <v>92</v>
       </c>
-      <c r="R20">
+      <c r="S20">
         <v>0.2</v>
       </c>
-      <c r="V20" s="2" t="s">
+      <c r="W20" s="2" t="s">
         <v>433</v>
       </c>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>32</v>
       </c>
@@ -3537,17 +3566,17 @@
       <c r="L21">
         <v>4.3999999999999997E-2</v>
       </c>
-      <c r="Q21">
+      <c r="R21">
         <v>31</v>
       </c>
-      <c r="R21">
+      <c r="S21">
         <v>6.8000000000000005E-2</v>
       </c>
-      <c r="V21" s="2" t="s">
+      <c r="W21" s="2" t="s">
         <v>432</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>33</v>
       </c>
@@ -3584,17 +3613,17 @@
       <c r="L22">
         <v>3.3000000000000002E-2</v>
       </c>
-      <c r="Q22">
+      <c r="R22">
         <v>20</v>
       </c>
-      <c r="R22">
+      <c r="S22">
         <v>4.3999999999999997E-2</v>
       </c>
-      <c r="V22" s="2" t="s">
+      <c r="W22" s="2" t="s">
         <v>485</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>34</v>
       </c>
@@ -3629,17 +3658,17 @@
       <c r="L23">
         <v>0.17199999999999999</v>
       </c>
-      <c r="Q23">
+      <c r="R23">
         <v>106</v>
       </c>
-      <c r="R23">
+      <c r="S23">
         <v>0.23100000000000001</v>
       </c>
-      <c r="V23" s="2" t="s">
+      <c r="W23" s="2" t="s">
         <v>431</v>
       </c>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>35</v>
       </c>
@@ -3674,17 +3703,17 @@
       <c r="L24">
         <v>8.1000000000000003E-2</v>
       </c>
-      <c r="Q24">
+      <c r="R24">
         <v>55</v>
       </c>
-      <c r="R24">
+      <c r="S24">
         <v>0.12</v>
       </c>
-      <c r="V24" s="2" t="s">
+      <c r="W24" s="2" t="s">
         <v>430</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>36</v>
       </c>
@@ -3719,17 +3748,17 @@
       <c r="L25">
         <v>0.126</v>
       </c>
-      <c r="Q25">
+      <c r="R25">
         <v>82</v>
       </c>
-      <c r="R25">
+      <c r="S25">
         <v>0.17899999999999999</v>
       </c>
-      <c r="V25" s="2" t="s">
+      <c r="W25" s="2" t="s">
         <v>429</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>37</v>
       </c>
@@ -3761,17 +3790,17 @@
       <c r="L26">
         <v>1E-3</v>
       </c>
-      <c r="Q26">
+      <c r="R26">
         <v>1</v>
       </c>
-      <c r="R26" s="4">
+      <c r="S26" s="4">
         <v>2E-3</v>
       </c>
-      <c r="V26" s="2" t="s">
+      <c r="W26" s="2" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>38</v>
       </c>
@@ -3809,20 +3838,20 @@
       <c r="O27" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q27">
+      <c r="R27">
         <v>13</v>
       </c>
-      <c r="R27">
+      <c r="S27">
         <v>2.8000000000000001E-2</v>
       </c>
-      <c r="S27" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V27" s="2" t="s">
+      <c r="T27" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W27" s="2" t="s">
         <v>428</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>39</v>
       </c>
@@ -3863,20 +3892,20 @@
       <c r="O28" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q28">
+      <c r="R28">
         <v>5</v>
       </c>
-      <c r="R28" s="4">
+      <c r="S28" s="4">
         <v>1.0999999999999999E-2</v>
       </c>
-      <c r="S28" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V28" s="2" t="s">
+      <c r="T28" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W28" s="2" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>40</v>
       </c>
@@ -3914,20 +3943,20 @@
       <c r="O29" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q29">
+      <c r="R29">
         <v>2</v>
       </c>
-      <c r="R29" s="4">
+      <c r="S29" s="4">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="S29" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V29" s="2" t="s">
+      <c r="T29" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W29" s="2" t="s">
         <v>426</v>
       </c>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>41</v>
       </c>
@@ -3967,20 +3996,20 @@
       <c r="O30" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q30">
+      <c r="R30">
         <v>23</v>
       </c>
-      <c r="R30">
+      <c r="S30">
         <v>0.05</v>
       </c>
-      <c r="S30" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V30" s="2" t="s">
+      <c r="T30" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W30" s="2" t="s">
         <v>425</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>42</v>
       </c>
@@ -4021,20 +4050,20 @@
       <c r="O31" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q31">
+      <c r="R31">
         <v>73</v>
       </c>
-      <c r="R31">
+      <c r="S31">
         <v>0.159</v>
       </c>
-      <c r="S31" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V31" s="2" t="s">
+      <c r="T31" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W31" s="2" t="s">
         <v>424</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>43</v>
       </c>
@@ -4075,20 +4104,20 @@
       <c r="O32" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q32">
+      <c r="R32">
         <v>68</v>
       </c>
-      <c r="R32">
+      <c r="S32">
         <v>0.14799999999999999</v>
       </c>
-      <c r="S32" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V32" s="2" t="s">
+      <c r="T32" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W32" s="2" t="s">
         <v>407</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>44</v>
       </c>
@@ -4134,26 +4163,29 @@
       <c r="O33" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="P33" t="s">
+      <c r="P33" s="10" t="s">
+        <v>511</v>
+      </c>
+      <c r="Q33" t="s">
         <v>43</v>
       </c>
-      <c r="Q33">
+      <c r="R33">
         <v>3</v>
       </c>
-      <c r="R33" s="4">
+      <c r="S33" s="4">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="S33" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="T33" t="s">
+      <c r="T33" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="U33" t="s">
         <v>43</v>
       </c>
-      <c r="V33" s="2" t="s">
+      <c r="W33" s="2" t="s">
         <v>407</v>
       </c>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>45</v>
       </c>
@@ -4196,20 +4228,20 @@
       <c r="O34" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q34">
+      <c r="R34">
         <v>23</v>
       </c>
-      <c r="R34">
+      <c r="S34">
         <v>0.05</v>
       </c>
-      <c r="S34" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V34" s="2" t="s">
+      <c r="T34" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W34" s="2" t="s">
         <v>409</v>
       </c>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>46</v>
       </c>
@@ -4248,21 +4280,21 @@
       <c r="O35" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q35">
-        <v>0</v>
-      </c>
       <c r="R35">
         <v>0</v>
       </c>
-      <c r="S35" s="8"/>
-      <c r="U35" t="s">
+      <c r="S35">
+        <v>0</v>
+      </c>
+      <c r="T35" s="8"/>
+      <c r="V35" t="s">
         <v>324</v>
       </c>
-      <c r="V35" s="2" t="s">
+      <c r="W35" s="2" t="s">
         <v>410</v>
       </c>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>47</v>
       </c>
@@ -4303,20 +4335,20 @@
       <c r="O36" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q36">
+      <c r="R36">
         <v>138</v>
       </c>
-      <c r="R36">
+      <c r="S36">
         <v>0.30099999999999999</v>
       </c>
-      <c r="S36" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V36" s="2" t="s">
+      <c r="T36" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W36" s="2" t="s">
         <v>411</v>
       </c>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>48</v>
       </c>
@@ -4357,20 +4389,20 @@
       <c r="O37" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q37">
+      <c r="R37">
         <v>45</v>
       </c>
-      <c r="R37">
+      <c r="S37">
         <v>9.8000000000000004E-2</v>
       </c>
-      <c r="S37" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V37" s="2" t="s">
+      <c r="T37" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W37" s="2" t="s">
         <v>412</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>49</v>
       </c>
@@ -4411,20 +4443,20 @@
       <c r="O38" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q38">
+      <c r="R38">
         <v>24</v>
       </c>
-      <c r="R38">
+      <c r="S38">
         <v>5.1999999999999998E-2</v>
       </c>
-      <c r="S38" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V38" s="2" t="s">
+      <c r="T38" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W38" s="2" t="s">
         <v>413</v>
       </c>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>50</v>
       </c>
@@ -4467,20 +4499,20 @@
       <c r="O39" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q39">
+      <c r="R39">
         <v>38</v>
       </c>
-      <c r="R39">
+      <c r="S39">
         <v>8.3000000000000004E-2</v>
       </c>
-      <c r="S39" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V39" s="2" t="s">
+      <c r="T39" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W39" s="2" t="s">
         <v>414</v>
       </c>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>51</v>
       </c>
@@ -4526,26 +4558,29 @@
       <c r="O40" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="P40" t="s">
+      <c r="P40" s="10" t="s">
+        <v>510</v>
+      </c>
+      <c r="Q40" t="s">
         <v>52</v>
       </c>
-      <c r="Q40">
+      <c r="R40">
         <v>12</v>
       </c>
-      <c r="R40">
+      <c r="S40">
         <v>2.5999999999999999E-2</v>
       </c>
-      <c r="S40" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="T40" t="s">
+      <c r="T40" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="U40" t="s">
         <v>52</v>
       </c>
-      <c r="V40" s="2" t="s">
+      <c r="W40" s="2" t="s">
         <v>416</v>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>52</v>
       </c>
@@ -4588,20 +4623,20 @@
       <c r="O41" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q41">
+      <c r="R41">
         <v>70</v>
       </c>
-      <c r="R41">
+      <c r="S41">
         <v>0.153</v>
       </c>
-      <c r="S41" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V41" s="2" t="s">
+      <c r="T41" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W41" s="2" t="s">
         <v>416</v>
       </c>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>53</v>
       </c>
@@ -4644,20 +4679,20 @@
       <c r="O42" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q42">
+      <c r="R42">
         <v>44</v>
       </c>
-      <c r="R42">
+      <c r="S42">
         <v>9.6000000000000002E-2</v>
       </c>
-      <c r="S42" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V42" s="2" t="s">
+      <c r="T42" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W42" s="2" t="s">
         <v>417</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>54</v>
       </c>
@@ -4700,20 +4735,20 @@
       <c r="O43" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q43">
+      <c r="R43">
         <v>8</v>
       </c>
-      <c r="R43">
+      <c r="S43">
         <v>1.7000000000000001E-2</v>
       </c>
-      <c r="S43" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V43" s="2" t="s">
+      <c r="T43" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W43" s="2" t="s">
         <v>491</v>
       </c>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>55</v>
       </c>
@@ -4759,26 +4794,29 @@
       <c r="O44" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="P44" t="s">
+      <c r="P44" s="10" t="s">
+        <v>590</v>
+      </c>
+      <c r="Q44" t="s">
         <v>54</v>
       </c>
-      <c r="Q44">
+      <c r="R44">
         <v>18</v>
       </c>
-      <c r="R44">
+      <c r="S44">
         <v>3.9E-2</v>
       </c>
-      <c r="S44" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="T44" t="s">
+      <c r="T44" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="U44" t="s">
         <v>54</v>
       </c>
-      <c r="V44" s="2" t="s">
+      <c r="W44" s="2" t="s">
         <v>491</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>56</v>
       </c>
@@ -4821,20 +4859,20 @@
       <c r="O45" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q45">
+      <c r="R45">
         <v>14</v>
       </c>
-      <c r="R45">
+      <c r="S45">
         <v>3.1E-2</v>
       </c>
-      <c r="S45" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V45" s="2" t="s">
+      <c r="T45" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W45" s="2" t="s">
         <v>420</v>
       </c>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>57</v>
       </c>
@@ -4873,21 +4911,21 @@
       <c r="O46" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q46">
-        <v>0</v>
-      </c>
       <c r="R46">
         <v>0</v>
       </c>
-      <c r="S46" s="8"/>
-      <c r="U46" t="s">
+      <c r="S46">
+        <v>0</v>
+      </c>
+      <c r="T46" s="8"/>
+      <c r="V46" t="s">
         <v>324</v>
       </c>
-      <c r="V46" s="2" t="s">
+      <c r="W46" s="2" t="s">
         <v>421</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>58</v>
       </c>
@@ -4928,20 +4966,20 @@
       <c r="O47" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q47">
+      <c r="R47">
         <v>258</v>
       </c>
-      <c r="R47">
+      <c r="S47">
         <v>0.56200000000000006</v>
       </c>
-      <c r="S47" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V47" s="2" t="s">
+      <c r="T47" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W47" s="2" t="s">
         <v>422</v>
       </c>
     </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>59</v>
       </c>
@@ -4984,20 +5022,20 @@
       <c r="O48" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q48">
+      <c r="R48">
         <v>85</v>
       </c>
-      <c r="R48">
+      <c r="S48">
         <v>0.185</v>
       </c>
-      <c r="S48" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V48" s="2" t="s">
+      <c r="T48" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W48" s="2" t="s">
         <v>423</v>
       </c>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>60</v>
       </c>
@@ -5040,20 +5078,20 @@
       <c r="O49" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q49">
+      <c r="R49">
         <v>14</v>
       </c>
-      <c r="R49">
+      <c r="S49">
         <v>3.1E-2</v>
       </c>
-      <c r="S49" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V49" s="2" t="s">
+      <c r="T49" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W49" s="2" t="s">
         <v>455</v>
       </c>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>61</v>
       </c>
@@ -5094,20 +5132,20 @@
       <c r="O50" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q50">
+      <c r="R50">
         <v>77</v>
       </c>
-      <c r="R50">
+      <c r="S50">
         <v>0.16800000000000001</v>
       </c>
-      <c r="S50" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V50" s="2" t="s">
+      <c r="T50" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W50" s="2" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>62</v>
       </c>
@@ -5135,17 +5173,17 @@
       <c r="L51">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="Q51">
+      <c r="R51">
         <v>4</v>
       </c>
-      <c r="R51">
+      <c r="S51">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="V51" s="2" t="s">
+      <c r="W51" s="2" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>63</v>
       </c>
@@ -5186,20 +5224,20 @@
       <c r="O52" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q52">
+      <c r="R52">
         <v>2</v>
       </c>
-      <c r="R52">
+      <c r="S52">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="S52" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V52" s="2" t="s">
+      <c r="T52" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W52" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>64</v>
       </c>
@@ -5233,17 +5271,17 @@
       <c r="L53">
         <v>0.14799999999999999</v>
       </c>
-      <c r="Q53">
+      <c r="R53">
         <v>93</v>
       </c>
-      <c r="R53">
+      <c r="S53">
         <v>0.20300000000000001</v>
       </c>
-      <c r="V53" s="2" t="s">
+      <c r="W53" s="2" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>65</v>
       </c>
@@ -5275,23 +5313,26 @@
       <c r="N54" t="s">
         <v>326</v>
       </c>
-      <c r="P54" t="s">
+      <c r="P54" s="10" t="s">
+        <v>656</v>
+      </c>
+      <c r="Q54" t="s">
         <v>326</v>
       </c>
-      <c r="Q54">
+      <c r="R54">
         <v>2</v>
       </c>
-      <c r="R54">
+      <c r="S54">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="T54" t="s">
+      <c r="U54" t="s">
         <v>326</v>
       </c>
-      <c r="V54" t="s">
+      <c r="W54" t="s">
         <v>492</v>
       </c>
     </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>66</v>
       </c>
@@ -5326,17 +5367,17 @@
       <c r="L55">
         <v>0.14799999999999999</v>
       </c>
-      <c r="Q55">
+      <c r="R55">
         <v>88</v>
       </c>
-      <c r="R55">
+      <c r="S55">
         <v>0.192</v>
       </c>
-      <c r="V55" s="2" t="s">
+      <c r="W55" s="2" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>67</v>
       </c>
@@ -5370,17 +5411,17 @@
       <c r="L56">
         <v>0.126</v>
       </c>
-      <c r="Q56">
+      <c r="R56">
         <v>85</v>
       </c>
-      <c r="R56">
+      <c r="S56">
         <v>0.185</v>
       </c>
-      <c r="V56" s="2" t="s">
+      <c r="W56" s="2" t="s">
         <v>406</v>
       </c>
     </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>68</v>
       </c>
@@ -5417,23 +5458,26 @@
       <c r="N57" t="s">
         <v>326</v>
       </c>
-      <c r="P57" t="s">
+      <c r="P57" s="10" t="s">
+        <v>656</v>
+      </c>
+      <c r="Q57" t="s">
         <v>326</v>
       </c>
-      <c r="Q57">
+      <c r="R57">
         <v>10</v>
       </c>
-      <c r="R57">
+      <c r="S57">
         <v>2.1999999999999999E-2</v>
       </c>
-      <c r="T57" t="s">
+      <c r="U57" t="s">
         <v>326</v>
       </c>
-      <c r="V57" s="2" t="s">
+      <c r="W57" s="2" t="s">
         <v>492</v>
       </c>
     </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>69</v>
       </c>
@@ -5465,23 +5509,26 @@
       <c r="N58" t="s">
         <v>326</v>
       </c>
-      <c r="P58" t="s">
+      <c r="P58" s="10" t="s">
+        <v>656</v>
+      </c>
+      <c r="Q58" t="s">
         <v>326</v>
       </c>
-      <c r="Q58">
+      <c r="R58">
         <v>8</v>
       </c>
-      <c r="R58">
+      <c r="S58">
         <v>1.7000000000000001E-2</v>
       </c>
-      <c r="T58" t="s">
+      <c r="U58" t="s">
         <v>326</v>
       </c>
-      <c r="V58" t="s">
+      <c r="W58" t="s">
         <v>492</v>
       </c>
     </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>70</v>
       </c>
@@ -5522,26 +5569,29 @@
       <c r="O59" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="P59" t="s">
+      <c r="P59" s="10" t="s">
+        <v>505</v>
+      </c>
+      <c r="Q59" t="s">
         <v>70</v>
       </c>
-      <c r="Q59">
+      <c r="R59">
         <v>5</v>
       </c>
-      <c r="R59">
+      <c r="S59">
         <v>1.0999999999999999E-2</v>
       </c>
-      <c r="S59" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="T59" t="s">
+      <c r="T59" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="U59" t="s">
         <v>70</v>
       </c>
-      <c r="V59" s="2" t="s">
+      <c r="W59" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>71</v>
       </c>
@@ -5585,26 +5635,29 @@
       <c r="O60" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="P60" t="s">
+      <c r="P60" s="10" t="s">
+        <v>505</v>
+      </c>
+      <c r="Q60" t="s">
         <v>70</v>
       </c>
-      <c r="Q60">
+      <c r="R60">
         <v>10</v>
       </c>
-      <c r="R60">
+      <c r="S60">
         <v>2.1999999999999999E-2</v>
       </c>
-      <c r="S60" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="T60" t="s">
+      <c r="T60" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="U60" t="s">
         <v>70</v>
       </c>
-      <c r="V60" s="2" t="s">
+      <c r="W60" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>72</v>
       </c>
@@ -5648,26 +5701,29 @@
       <c r="O61" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="P61" t="s">
+      <c r="P61" s="10" t="s">
+        <v>505</v>
+      </c>
+      <c r="Q61" t="s">
         <v>70</v>
       </c>
-      <c r="Q61">
+      <c r="R61">
         <v>2</v>
       </c>
-      <c r="R61">
+      <c r="S61">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="S61" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="T61" t="s">
+      <c r="T61" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="U61" t="s">
         <v>70</v>
       </c>
-      <c r="V61" s="2" t="s">
+      <c r="W61" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>73</v>
       </c>
@@ -5711,23 +5767,26 @@
       <c r="O62" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="P62" t="s">
+      <c r="P62" s="10" t="s">
+        <v>657</v>
+      </c>
+      <c r="Q62" t="s">
         <v>256</v>
       </c>
-      <c r="Q62">
+      <c r="R62">
         <v>7</v>
       </c>
-      <c r="R62">
+      <c r="S62">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="S62" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V62" t="s">
+      <c r="T62" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W62" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>74</v>
       </c>
@@ -5771,23 +5830,26 @@
       <c r="O63" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="P63" t="s">
+      <c r="P63" s="10" t="s">
+        <v>657</v>
+      </c>
+      <c r="Q63" t="s">
         <v>256</v>
       </c>
-      <c r="Q63">
+      <c r="R63">
         <v>14</v>
       </c>
-      <c r="R63">
+      <c r="S63">
         <v>3.1E-2</v>
       </c>
-      <c r="S63" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V63" t="s">
+      <c r="T63" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W63" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>75</v>
       </c>
@@ -5831,23 +5893,26 @@
       <c r="O64" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="P64" t="s">
+      <c r="P64" s="10" t="s">
+        <v>657</v>
+      </c>
+      <c r="Q64" t="s">
         <v>256</v>
       </c>
-      <c r="Q64">
+      <c r="R64">
         <v>4</v>
       </c>
-      <c r="R64">
+      <c r="S64">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="S64" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V64" t="s">
+      <c r="T64" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W64" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>76</v>
       </c>
@@ -5891,26 +5956,29 @@
       <c r="O65" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="P65" t="s">
+      <c r="P65" s="10" t="s">
+        <v>657</v>
+      </c>
+      <c r="Q65" t="s">
         <v>256</v>
       </c>
-      <c r="Q65">
+      <c r="R65">
         <v>3</v>
       </c>
-      <c r="R65">
+      <c r="S65">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="S65" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="T65" t="s">
+      <c r="T65" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="U65" t="s">
         <v>330</v>
       </c>
-      <c r="V65" t="s">
+      <c r="W65" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>77</v>
       </c>
@@ -5954,26 +6022,29 @@
       <c r="O66" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="P66" t="s">
+      <c r="P66" s="10" t="s">
+        <v>657</v>
+      </c>
+      <c r="Q66" t="s">
         <v>256</v>
       </c>
-      <c r="Q66">
+      <c r="R66">
         <v>13</v>
       </c>
-      <c r="R66">
+      <c r="S66">
         <v>2.8000000000000001E-2</v>
       </c>
-      <c r="S66" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="T66" t="s">
+      <c r="T66" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="U66" t="s">
         <v>330</v>
       </c>
-      <c r="V66" t="s">
+      <c r="W66" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>78</v>
       </c>
@@ -6019,26 +6090,29 @@
       <c r="O67" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="P67" t="s">
+      <c r="P67" s="10" t="s">
+        <v>657</v>
+      </c>
+      <c r="Q67" t="s">
         <v>256</v>
       </c>
-      <c r="Q67">
+      <c r="R67">
         <v>3</v>
       </c>
-      <c r="R67">
+      <c r="S67">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="S67" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="T67" t="s">
+      <c r="T67" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="U67" t="s">
         <v>330</v>
       </c>
-      <c r="V67" t="s">
+      <c r="W67" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="68" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>79</v>
       </c>
@@ -6068,23 +6142,26 @@
       <c r="N68" t="s">
         <v>79</v>
       </c>
-      <c r="P68" t="s">
+      <c r="P68" s="10" t="s">
+        <v>553</v>
+      </c>
+      <c r="Q68" t="s">
         <v>79</v>
       </c>
-      <c r="Q68">
+      <c r="R68">
         <v>294</v>
       </c>
-      <c r="R68">
+      <c r="S68">
         <v>0.64100000000000001</v>
       </c>
-      <c r="T68" t="s">
+      <c r="U68" t="s">
         <v>79</v>
       </c>
-      <c r="V68" s="2" t="s">
+      <c r="W68" s="2" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>80</v>
       </c>
@@ -6116,23 +6193,26 @@
       <c r="N69" t="s">
         <v>79</v>
       </c>
-      <c r="P69" t="s">
+      <c r="P69" s="10" t="s">
+        <v>553</v>
+      </c>
+      <c r="Q69" t="s">
         <v>79</v>
       </c>
-      <c r="Q69">
+      <c r="R69">
         <v>128</v>
       </c>
-      <c r="R69">
+      <c r="S69">
         <v>0.27900000000000003</v>
       </c>
-      <c r="T69" t="s">
+      <c r="U69" t="s">
         <v>79</v>
       </c>
-      <c r="V69" s="2" t="s">
+      <c r="W69" s="2" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>81</v>
       </c>
@@ -6164,23 +6244,26 @@
       <c r="N70" t="s">
         <v>79</v>
       </c>
-      <c r="P70" t="s">
+      <c r="P70" s="10" t="s">
+        <v>553</v>
+      </c>
+      <c r="Q70" t="s">
         <v>79</v>
       </c>
-      <c r="Q70">
+      <c r="R70">
         <v>57</v>
       </c>
-      <c r="R70">
+      <c r="S70">
         <v>0.124</v>
       </c>
-      <c r="T70" t="s">
+      <c r="U70" t="s">
         <v>79</v>
       </c>
-      <c r="V70" s="2" t="s">
+      <c r="W70" s="2" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>82</v>
       </c>
@@ -6212,23 +6295,26 @@
       <c r="N71" t="s">
         <v>15</v>
       </c>
-      <c r="P71" t="s">
+      <c r="P71" s="11" t="s">
+        <v>566</v>
+      </c>
+      <c r="Q71" t="s">
         <v>15</v>
       </c>
-      <c r="Q71">
+      <c r="R71">
         <v>7</v>
       </c>
-      <c r="R71">
+      <c r="S71">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="T71" t="s">
+      <c r="U71" t="s">
         <v>15</v>
       </c>
-      <c r="V71" s="2" t="s">
+      <c r="W71" s="2" t="s">
         <v>447</v>
       </c>
     </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>83</v>
       </c>
@@ -6257,17 +6343,17 @@
       <c r="L72">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="Q72">
+      <c r="R72">
         <v>58</v>
       </c>
-      <c r="R72">
+      <c r="S72">
         <v>0.126</v>
       </c>
-      <c r="V72" s="2" t="s">
+      <c r="W72" s="2" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>84</v>
       </c>
@@ -6299,23 +6385,26 @@
       <c r="N73" t="s">
         <v>79</v>
       </c>
-      <c r="P73" t="s">
+      <c r="P73" s="10" t="s">
+        <v>553</v>
+      </c>
+      <c r="Q73" t="s">
         <v>79</v>
       </c>
-      <c r="Q73">
+      <c r="R73">
         <v>12</v>
       </c>
-      <c r="R73">
+      <c r="S73">
         <v>2.5999999999999999E-2</v>
       </c>
-      <c r="T73" t="s">
+      <c r="U73" t="s">
         <v>79</v>
       </c>
-      <c r="V73" s="2" t="s">
+      <c r="W73" s="2" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="74" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>85</v>
       </c>
@@ -6347,23 +6436,26 @@
       <c r="N74" t="s">
         <v>79</v>
       </c>
-      <c r="P74" t="s">
+      <c r="P74" s="10" t="s">
+        <v>553</v>
+      </c>
+      <c r="Q74" t="s">
         <v>79</v>
       </c>
-      <c r="Q74">
+      <c r="R74">
         <v>15</v>
       </c>
-      <c r="R74">
+      <c r="S74">
         <v>3.3000000000000002E-2</v>
       </c>
-      <c r="T74" t="s">
+      <c r="U74" t="s">
         <v>79</v>
       </c>
-      <c r="V74" s="2" t="s">
+      <c r="W74" s="2" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>86</v>
       </c>
@@ -6395,23 +6487,26 @@
       <c r="N75" t="s">
         <v>79</v>
       </c>
-      <c r="P75" t="s">
+      <c r="P75" s="10" t="s">
+        <v>553</v>
+      </c>
+      <c r="Q75" t="s">
         <v>79</v>
       </c>
-      <c r="Q75">
+      <c r="R75">
         <v>18</v>
       </c>
-      <c r="R75">
+      <c r="S75">
         <v>3.9E-2</v>
       </c>
-      <c r="T75" t="s">
+      <c r="U75" t="s">
         <v>79</v>
       </c>
-      <c r="V75" s="2" t="s">
+      <c r="W75" s="2" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>87</v>
       </c>
@@ -6446,17 +6541,17 @@
       <c r="L76">
         <v>3.5999999999999997E-2</v>
       </c>
-      <c r="Q76">
+      <c r="R76">
         <v>26</v>
       </c>
-      <c r="R76">
+      <c r="S76">
         <v>5.7000000000000002E-2</v>
       </c>
-      <c r="V76" s="2" t="s">
+      <c r="W76" s="2" t="s">
         <v>401</v>
       </c>
     </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>88</v>
       </c>
@@ -6493,23 +6588,26 @@
       <c r="N77" t="s">
         <v>87</v>
       </c>
-      <c r="P77" t="s">
+      <c r="P77" s="10" t="s">
+        <v>544</v>
+      </c>
+      <c r="Q77" t="s">
         <v>87</v>
       </c>
-      <c r="Q77">
+      <c r="R77">
         <v>2</v>
       </c>
-      <c r="R77">
+      <c r="S77">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="T77" t="s">
+      <c r="U77" t="s">
         <v>87</v>
       </c>
-      <c r="V77" t="s">
+      <c r="W77" t="s">
         <v>401</v>
       </c>
     </row>
-    <row r="78" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>89</v>
       </c>
@@ -6547,20 +6645,23 @@
       <c r="N78" t="s">
         <v>327</v>
       </c>
-      <c r="P78" t="s">
+      <c r="P78" s="10" t="s">
+        <v>658</v>
+      </c>
+      <c r="Q78" t="s">
         <v>327</v>
       </c>
-      <c r="Q78">
+      <c r="R78">
         <v>13</v>
       </c>
-      <c r="R78">
+      <c r="S78">
         <v>2.8000000000000001E-2</v>
       </c>
-      <c r="V78" s="2" t="s">
+      <c r="W78" s="2" t="s">
         <v>493</v>
       </c>
     </row>
-    <row r="79" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>90</v>
       </c>
@@ -6598,20 +6699,23 @@
       <c r="N79" t="s">
         <v>327</v>
       </c>
-      <c r="P79" t="s">
+      <c r="P79" s="10" t="s">
+        <v>658</v>
+      </c>
+      <c r="Q79" t="s">
         <v>327</v>
       </c>
-      <c r="Q79">
+      <c r="R79">
         <v>116</v>
       </c>
-      <c r="R79">
+      <c r="S79">
         <v>0.253</v>
       </c>
-      <c r="V79" s="2" t="s">
+      <c r="W79" s="2" t="s">
         <v>493</v>
       </c>
     </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>91</v>
       </c>
@@ -6648,23 +6752,26 @@
       <c r="N80" t="s">
         <v>87</v>
       </c>
-      <c r="P80" t="s">
+      <c r="P80" s="10" t="s">
+        <v>544</v>
+      </c>
+      <c r="Q80" t="s">
         <v>87</v>
       </c>
-      <c r="Q80">
+      <c r="R80">
         <v>7</v>
       </c>
-      <c r="R80">
+      <c r="S80">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="T80" t="s">
+      <c r="U80" t="s">
         <v>87</v>
       </c>
-      <c r="V80" t="s">
+      <c r="W80" t="s">
         <v>401</v>
       </c>
     </row>
-    <row r="81" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>92</v>
       </c>
@@ -6699,17 +6806,17 @@
       <c r="L81">
         <v>2.1000000000000001E-2</v>
       </c>
-      <c r="Q81">
+      <c r="R81">
         <v>18</v>
       </c>
-      <c r="R81">
+      <c r="S81">
         <v>3.9E-2</v>
       </c>
-      <c r="V81" t="s">
+      <c r="W81" t="s">
         <v>396</v>
       </c>
     </row>
-    <row r="82" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>93</v>
       </c>
@@ -6744,17 +6851,17 @@
       <c r="L82">
         <v>3.4000000000000002E-2</v>
       </c>
-      <c r="Q82">
+      <c r="R82">
         <v>23</v>
       </c>
-      <c r="R82">
+      <c r="S82">
         <v>0.05</v>
       </c>
-      <c r="V82" s="2" t="s">
+      <c r="W82" s="2" t="s">
         <v>395</v>
       </c>
     </row>
-    <row r="83" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>94</v>
       </c>
@@ -6792,23 +6899,26 @@
       <c r="N83" t="s">
         <v>328</v>
       </c>
-      <c r="P83" t="s">
+      <c r="P83" s="10" t="s">
+        <v>551</v>
+      </c>
+      <c r="Q83" t="s">
         <v>328</v>
       </c>
-      <c r="Q83">
+      <c r="R83">
         <v>12</v>
       </c>
-      <c r="R83">
+      <c r="S83">
         <v>2.5999999999999999E-2</v>
       </c>
-      <c r="T83" t="s">
+      <c r="U83" t="s">
         <v>328</v>
       </c>
-      <c r="V83" t="s">
+      <c r="W83" t="s">
         <v>494</v>
       </c>
     </row>
-    <row r="84" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>95</v>
       </c>
@@ -6846,23 +6956,26 @@
       <c r="N84" t="s">
         <v>328</v>
       </c>
-      <c r="P84" t="s">
+      <c r="P84" s="10" t="s">
+        <v>551</v>
+      </c>
+      <c r="Q84" t="s">
         <v>328</v>
       </c>
-      <c r="Q84">
+      <c r="R84">
         <v>9</v>
       </c>
-      <c r="R84">
+      <c r="S84">
         <v>0.02</v>
       </c>
-      <c r="T84" t="s">
+      <c r="U84" t="s">
         <v>328</v>
       </c>
-      <c r="V84" t="s">
+      <c r="W84" t="s">
         <v>494</v>
       </c>
     </row>
-    <row r="85" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>96</v>
       </c>
@@ -6897,17 +7010,17 @@
       <c r="L85">
         <v>2.3E-2</v>
       </c>
-      <c r="Q85">
+      <c r="R85">
         <v>19</v>
       </c>
-      <c r="R85">
+      <c r="S85">
         <v>4.1000000000000002E-2</v>
       </c>
-      <c r="V85" s="2" t="s">
+      <c r="W85" s="2" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="86" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>97</v>
       </c>
@@ -6941,17 +7054,17 @@
       <c r="L86">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="Q86">
+      <c r="R86">
         <v>28</v>
       </c>
-      <c r="R86">
+      <c r="S86">
         <v>6.0999999999999999E-2</v>
       </c>
-      <c r="V86" s="2" t="s">
+      <c r="W86" s="2" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="87" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>98</v>
       </c>
@@ -6986,17 +7099,17 @@
       <c r="L87">
         <v>9.5000000000000001E-2</v>
       </c>
-      <c r="Q87">
+      <c r="R87">
         <v>66</v>
       </c>
-      <c r="R87">
+      <c r="S87">
         <v>0.14399999999999999</v>
       </c>
-      <c r="V87" s="2" t="s">
+      <c r="W87" s="2" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="88" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>99</v>
       </c>
@@ -7034,20 +7147,20 @@
       <c r="O88" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q88">
+      <c r="R88">
         <v>53</v>
       </c>
-      <c r="R88">
+      <c r="S88">
         <v>0.115</v>
       </c>
-      <c r="S88" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V88" s="2" t="s">
+      <c r="T88" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W88" s="2" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="89" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>100</v>
       </c>
@@ -7088,20 +7201,20 @@
       <c r="O89" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q89">
+      <c r="R89">
         <v>1</v>
       </c>
-      <c r="R89">
+      <c r="S89">
         <v>2E-3</v>
       </c>
-      <c r="S89" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V89" s="2" t="s">
+      <c r="T89" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W89" s="2" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="90" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>101</v>
       </c>
@@ -7136,17 +7249,17 @@
       <c r="L90">
         <v>0.189</v>
       </c>
-      <c r="Q90">
+      <c r="R90">
         <v>128</v>
       </c>
-      <c r="R90">
+      <c r="S90">
         <v>0.27900000000000003</v>
       </c>
-      <c r="V90" s="2" t="s">
+      <c r="W90" s="2" t="s">
         <v>390</v>
       </c>
     </row>
-    <row r="91" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>102</v>
       </c>
@@ -7159,13 +7272,13 @@
       <c r="D91" s="2" t="s">
         <v>389</v>
       </c>
-      <c r="E91" s="19" t="s">
+      <c r="E91" s="10" t="s">
         <v>651</v>
       </c>
-      <c r="F91" s="19" t="s">
+      <c r="F91" s="10" t="s">
         <v>651</v>
       </c>
-      <c r="G91" s="20">
+      <c r="G91" s="2">
         <v>28447</v>
       </c>
       <c r="H91" s="3" t="s">
@@ -7186,23 +7299,26 @@
       <c r="N91" t="s">
         <v>101</v>
       </c>
-      <c r="P91" t="s">
+      <c r="P91" s="20" t="s">
+        <v>538</v>
+      </c>
+      <c r="Q91" t="s">
         <v>101</v>
       </c>
-      <c r="Q91">
+      <c r="R91">
         <v>8</v>
       </c>
-      <c r="R91">
+      <c r="S91">
         <v>1.7000000000000001E-2</v>
       </c>
-      <c r="T91" t="s">
+      <c r="U91" t="s">
         <v>101</v>
       </c>
-      <c r="V91" s="2" t="s">
+      <c r="W91" s="2" t="s">
         <v>390</v>
       </c>
     </row>
-    <row r="92" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>103</v>
       </c>
@@ -7215,7 +7331,7 @@
       <c r="D92" s="2" t="s">
         <v>388</v>
       </c>
-      <c r="E92" s="19"/>
+      <c r="E92" s="10"/>
       <c r="F92" s="15" t="s">
         <v>538</v>
       </c>
@@ -7237,17 +7353,17 @@
       <c r="L92">
         <v>8.6999999999999994E-2</v>
       </c>
-      <c r="Q92">
+      <c r="R92">
         <v>68</v>
       </c>
-      <c r="R92">
+      <c r="S92">
         <v>0.14799999999999999</v>
       </c>
-      <c r="V92" s="2" t="s">
+      <c r="W92" s="2" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="93" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>104</v>
       </c>
@@ -7282,20 +7398,20 @@
       <c r="L93">
         <v>2.9000000000000001E-2</v>
       </c>
-      <c r="P93" t="s">
+      <c r="Q93" t="s">
         <v>101</v>
       </c>
-      <c r="Q93">
+      <c r="R93">
         <v>24</v>
       </c>
-      <c r="R93">
+      <c r="S93">
         <v>5.1999999999999998E-2</v>
       </c>
-      <c r="V93" s="2" t="s">
+      <c r="W93" s="2" t="s">
         <v>495</v>
       </c>
     </row>
-    <row r="94" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>105</v>
       </c>
@@ -7332,17 +7448,17 @@
       <c r="L94">
         <v>0.105</v>
       </c>
-      <c r="Q94">
+      <c r="R94">
         <v>81</v>
       </c>
-      <c r="R94">
+      <c r="S94">
         <v>0.17599999999999999</v>
       </c>
-      <c r="V94" s="2" t="s">
+      <c r="W94" s="2" t="s">
         <v>496</v>
       </c>
     </row>
-    <row r="95" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>106</v>
       </c>
@@ -7379,20 +7495,20 @@
       <c r="L95">
         <v>2.1000000000000001E-2</v>
       </c>
-      <c r="P95" t="s">
+      <c r="Q95" t="s">
         <v>105</v>
       </c>
-      <c r="Q95">
+      <c r="R95">
         <v>17</v>
       </c>
-      <c r="R95">
+      <c r="S95">
         <v>3.6999999999999998E-2</v>
       </c>
-      <c r="V95" s="2" t="s">
+      <c r="W95" s="2" t="s">
         <v>496</v>
       </c>
     </row>
-    <row r="96" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>107</v>
       </c>
@@ -7429,17 +7545,17 @@
       <c r="L96">
         <v>5.6000000000000001E-2</v>
       </c>
-      <c r="Q96">
+      <c r="R96">
         <v>43</v>
       </c>
-      <c r="R96">
+      <c r="S96">
         <v>9.4E-2</v>
       </c>
-      <c r="V96" s="2" t="s">
+      <c r="W96" s="2" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="97" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>108</v>
       </c>
@@ -7476,17 +7592,17 @@
       <c r="L97">
         <v>8.5000000000000006E-2</v>
       </c>
-      <c r="Q97">
+      <c r="R97">
         <v>65</v>
       </c>
-      <c r="R97">
+      <c r="S97">
         <v>0.14199999999999999</v>
       </c>
-      <c r="V97" s="2" t="s">
+      <c r="W97" s="2" t="s">
         <v>383</v>
       </c>
     </row>
-    <row r="98" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:23" ht="30" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>109</v>
       </c>
@@ -7523,23 +7639,26 @@
       <c r="N98" t="s">
         <v>123</v>
       </c>
-      <c r="P98" t="s">
+      <c r="P98" s="10" t="s">
+        <v>543</v>
+      </c>
+      <c r="Q98" t="s">
         <v>123</v>
       </c>
-      <c r="Q98">
+      <c r="R98">
         <v>7</v>
       </c>
-      <c r="R98">
+      <c r="S98">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="T98" t="s">
+      <c r="U98" t="s">
         <v>123</v>
       </c>
-      <c r="V98" s="2" t="s">
+      <c r="W98" s="2" t="s">
         <v>368</v>
       </c>
     </row>
-    <row r="99" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>110</v>
       </c>
@@ -7576,17 +7695,17 @@
       <c r="L99">
         <v>4.5999999999999999E-2</v>
       </c>
-      <c r="Q99">
+      <c r="R99">
         <v>34</v>
       </c>
-      <c r="R99">
+      <c r="S99">
         <v>7.3999999999999996E-2</v>
       </c>
-      <c r="V99" s="2" t="s">
+      <c r="W99" s="2" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="100" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>111</v>
       </c>
@@ -7621,17 +7740,17 @@
       <c r="L100">
         <v>0.05</v>
       </c>
-      <c r="Q100">
+      <c r="R100">
         <v>37</v>
       </c>
-      <c r="R100">
+      <c r="S100">
         <v>8.1000000000000003E-2</v>
       </c>
-      <c r="V100" s="2" t="s">
+      <c r="W100" s="2" t="s">
         <v>380</v>
       </c>
     </row>
-    <row r="101" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>112</v>
       </c>
@@ -7669,23 +7788,26 @@
       <c r="N101" t="s">
         <v>101</v>
       </c>
-      <c r="P101" t="s">
+      <c r="P101" s="20" t="s">
+        <v>538</v>
+      </c>
+      <c r="Q101" t="s">
         <v>101</v>
       </c>
-      <c r="Q101">
+      <c r="R101">
         <v>6</v>
       </c>
-      <c r="R101">
+      <c r="S101">
         <v>1.2999999999999999E-2</v>
       </c>
-      <c r="T101" t="s">
+      <c r="U101" t="s">
         <v>101</v>
       </c>
-      <c r="V101" s="2" t="s">
+      <c r="W101" s="2" t="s">
         <v>390</v>
       </c>
     </row>
-    <row r="102" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>113</v>
       </c>
@@ -7720,17 +7842,17 @@
       <c r="L102">
         <v>0.03</v>
       </c>
-      <c r="Q102">
+      <c r="R102">
         <v>27</v>
       </c>
-      <c r="R102">
+      <c r="S102">
         <v>5.8999999999999997E-2</v>
       </c>
-      <c r="V102" s="2" t="s">
+      <c r="W102" s="2" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="103" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>114</v>
       </c>
@@ -7765,17 +7887,17 @@
       <c r="L103">
         <v>0.189</v>
       </c>
-      <c r="Q103">
+      <c r="R103">
         <v>121</v>
       </c>
-      <c r="R103">
+      <c r="S103">
         <v>0.26400000000000001</v>
       </c>
-      <c r="V103" s="2" t="s">
+      <c r="W103" s="2" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="104" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>115</v>
       </c>
@@ -7815,20 +7937,23 @@
       <c r="N104" t="s">
         <v>329</v>
       </c>
-      <c r="P104" t="s">
+      <c r="P104" s="10" t="s">
+        <v>659</v>
+      </c>
+      <c r="Q104" t="s">
         <v>329</v>
       </c>
-      <c r="Q104">
+      <c r="R104">
         <v>10</v>
       </c>
-      <c r="R104">
+      <c r="S104">
         <v>2.1999999999999999E-2</v>
       </c>
-      <c r="V104" s="2" t="s">
+      <c r="W104" s="2" t="s">
         <v>497</v>
       </c>
     </row>
-    <row r="105" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>116</v>
       </c>
@@ -7863,17 +7988,17 @@
       <c r="L105">
         <v>6.0999999999999999E-2</v>
       </c>
-      <c r="Q105">
+      <c r="R105">
         <v>40</v>
       </c>
-      <c r="R105">
+      <c r="S105">
         <v>8.6999999999999994E-2</v>
       </c>
-      <c r="V105" s="2" t="s">
+      <c r="W105" s="2" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="106" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>117</v>
       </c>
@@ -7908,17 +8033,17 @@
       <c r="L106">
         <v>5.8999999999999997E-2</v>
       </c>
-      <c r="Q106">
+      <c r="R106">
         <v>42</v>
       </c>
-      <c r="R106">
+      <c r="S106">
         <v>9.1999999999999998E-2</v>
       </c>
-      <c r="V106" s="2" t="s">
+      <c r="W106" s="2" t="s">
         <v>374</v>
       </c>
     </row>
-    <row r="107" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>118</v>
       </c>
@@ -7956,23 +8081,26 @@
       <c r="N107" t="s">
         <v>117</v>
       </c>
-      <c r="P107" t="s">
+      <c r="P107" s="10" t="s">
+        <v>534</v>
+      </c>
+      <c r="Q107" t="s">
         <v>117</v>
       </c>
-      <c r="Q107">
+      <c r="R107">
         <v>3</v>
       </c>
-      <c r="R107">
+      <c r="S107">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="T107" t="s">
+      <c r="U107" t="s">
         <v>117</v>
       </c>
-      <c r="V107" s="2" t="s">
+      <c r="W107" s="2" t="s">
         <v>374</v>
       </c>
     </row>
-    <row r="108" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>119</v>
       </c>
@@ -8010,20 +8138,23 @@
       <c r="N108" t="s">
         <v>329</v>
       </c>
-      <c r="P108" t="s">
+      <c r="P108" s="10" t="s">
+        <v>659</v>
+      </c>
+      <c r="Q108" t="s">
         <v>329</v>
       </c>
-      <c r="Q108">
+      <c r="R108">
         <v>11</v>
       </c>
-      <c r="R108">
+      <c r="S108">
         <v>2.4E-2</v>
       </c>
-      <c r="V108" s="2" t="s">
+      <c r="W108" s="2" t="s">
         <v>497</v>
       </c>
     </row>
-    <row r="109" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>120</v>
       </c>
@@ -8061,20 +8192,23 @@
       <c r="N109" t="s">
         <v>329</v>
       </c>
-      <c r="P109" t="s">
+      <c r="P109" s="10" t="s">
+        <v>659</v>
+      </c>
+      <c r="Q109" t="s">
         <v>329</v>
       </c>
-      <c r="Q109">
+      <c r="R109">
         <v>10</v>
       </c>
-      <c r="R109">
+      <c r="S109">
         <v>2.1999999999999999E-2</v>
       </c>
-      <c r="V109" s="2" t="s">
+      <c r="W109" s="2" t="s">
         <v>497</v>
       </c>
     </row>
-    <row r="110" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>121</v>
       </c>
@@ -8109,17 +8243,17 @@
       <c r="L110">
         <v>9.9000000000000005E-2</v>
       </c>
-      <c r="Q110">
+      <c r="R110">
         <v>67</v>
       </c>
-      <c r="R110">
+      <c r="S110">
         <v>0.14599999999999999</v>
       </c>
-      <c r="V110" s="2" t="s">
+      <c r="W110" s="2" t="s">
         <v>370</v>
       </c>
     </row>
-    <row r="111" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>122</v>
       </c>
@@ -8156,17 +8290,17 @@
       <c r="L111">
         <v>4.3999999999999997E-2</v>
       </c>
-      <c r="Q111">
+      <c r="R111">
         <v>31</v>
       </c>
-      <c r="R111">
+      <c r="S111">
         <v>6.8000000000000005E-2</v>
       </c>
-      <c r="V111" s="2" t="s">
+      <c r="W111" s="2" t="s">
         <v>369</v>
       </c>
     </row>
-    <row r="112" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>123</v>
       </c>
@@ -8201,17 +8335,17 @@
       <c r="L112">
         <v>3.9E-2</v>
       </c>
-      <c r="Q112">
+      <c r="R112">
         <v>30</v>
       </c>
-      <c r="R112">
+      <c r="S112">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="V112" s="2" t="s">
+      <c r="W112" s="2" t="s">
         <v>368</v>
       </c>
     </row>
-    <row r="113" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>124</v>
       </c>
@@ -8240,17 +8374,17 @@
       <c r="L113">
         <v>3.6999999999999998E-2</v>
       </c>
-      <c r="Q113">
+      <c r="R113">
         <v>29</v>
       </c>
-      <c r="R113">
+      <c r="S113">
         <v>6.3E-2</v>
       </c>
-      <c r="V113" s="2" t="s">
+      <c r="W113" s="2" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="114" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>125</v>
       </c>
@@ -8279,17 +8413,17 @@
       <c r="L114">
         <v>5.0999999999999997E-2</v>
       </c>
-      <c r="Q114">
+      <c r="R114">
         <v>45</v>
       </c>
-      <c r="R114">
+      <c r="S114">
         <v>9.8000000000000004E-2</v>
       </c>
-      <c r="V114" s="2" t="s">
+      <c r="W114" s="2" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="115" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>126</v>
       </c>
@@ -8324,17 +8458,17 @@
       <c r="L115">
         <v>5.7000000000000002E-2</v>
       </c>
-      <c r="Q115">
+      <c r="R115">
         <v>42</v>
       </c>
-      <c r="R115">
+      <c r="S115">
         <v>9.1999999999999998E-2</v>
       </c>
-      <c r="V115" s="2" t="s">
+      <c r="W115" s="2" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="116" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>127</v>
       </c>
@@ -8369,17 +8503,17 @@
       <c r="L116">
         <v>0.47299999999999998</v>
       </c>
-      <c r="Q116">
+      <c r="R116">
         <v>266</v>
       </c>
-      <c r="R116">
+      <c r="S116">
         <v>0.57999999999999996</v>
       </c>
-      <c r="V116" s="2" t="s">
+      <c r="W116" s="2" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="117" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>128</v>
       </c>
@@ -8417,20 +8551,23 @@
       <c r="N117" t="s">
         <v>127</v>
       </c>
-      <c r="P117" t="s">
+      <c r="P117" s="11" t="s">
+        <v>556</v>
+      </c>
+      <c r="Q117" t="s">
         <v>127</v>
       </c>
-      <c r="Q117">
+      <c r="R117">
         <v>15</v>
       </c>
-      <c r="R117">
+      <c r="S117">
         <v>3.3000000000000002E-2</v>
       </c>
-      <c r="V117" s="2" t="s">
+      <c r="W117" s="2" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="118" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>129</v>
       </c>
@@ -8465,17 +8602,17 @@
       <c r="L118">
         <v>0.21099999999999999</v>
       </c>
-      <c r="Q118">
+      <c r="R118">
         <v>135</v>
       </c>
-      <c r="R118">
+      <c r="S118">
         <v>0.29399999999999998</v>
       </c>
-      <c r="V118" s="2" t="s">
+      <c r="W118" s="2" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="119" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>130</v>
       </c>
@@ -8512,17 +8649,17 @@
       <c r="L119">
         <v>0.14699999999999999</v>
       </c>
-      <c r="Q119">
+      <c r="R119">
         <v>93</v>
       </c>
-      <c r="R119">
+      <c r="S119">
         <v>0.20300000000000001</v>
       </c>
-      <c r="V119" s="2" t="s">
+      <c r="W119" s="2" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="120" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>131</v>
       </c>
@@ -8557,17 +8694,17 @@
       <c r="L120">
         <v>0.35799999999999998</v>
       </c>
-      <c r="Q120">
+      <c r="R120">
         <v>211</v>
       </c>
-      <c r="R120">
+      <c r="S120">
         <v>0.46</v>
       </c>
-      <c r="V120" s="2" t="s">
+      <c r="W120" s="2" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="121" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>132</v>
       </c>
@@ -8602,17 +8739,17 @@
       <c r="L121">
         <v>0.81699999999999995</v>
       </c>
-      <c r="Q121">
+      <c r="R121">
         <v>380</v>
       </c>
-      <c r="R121">
+      <c r="S121">
         <v>0.82799999999999996</v>
       </c>
-      <c r="V121" s="2" t="s">
+      <c r="W121" s="2" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="122" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>133</v>
       </c>
@@ -8647,17 +8784,17 @@
       <c r="L122">
         <v>0.64</v>
       </c>
-      <c r="Q122">
+      <c r="R122">
         <v>340</v>
       </c>
-      <c r="R122">
+      <c r="S122">
         <v>0.74099999999999999</v>
       </c>
-      <c r="V122" s="2" t="s">
+      <c r="W122" s="2" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="123" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>134</v>
       </c>
@@ -8692,17 +8829,17 @@
       <c r="L123">
         <v>7.9000000000000001E-2</v>
       </c>
-      <c r="Q123">
+      <c r="R123">
         <v>49</v>
       </c>
-      <c r="R123">
+      <c r="S123">
         <v>0.107</v>
       </c>
-      <c r="V123" s="2" t="s">
+      <c r="W123" s="2" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="124" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>135</v>
       </c>
@@ -8729,17 +8866,17 @@
       <c r="L124">
         <v>0.33</v>
       </c>
-      <c r="Q124">
+      <c r="R124">
         <v>191</v>
       </c>
-      <c r="R124">
+      <c r="S124">
         <v>0.41599999999999998</v>
       </c>
-      <c r="V124" s="2" t="s">
+      <c r="W124" s="2" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="125" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>136</v>
       </c>
@@ -8766,17 +8903,17 @@
       <c r="L125">
         <v>7.6999999999999999E-2</v>
       </c>
-      <c r="Q125">
+      <c r="R125">
         <v>44</v>
       </c>
-      <c r="R125">
+      <c r="S125">
         <v>9.6000000000000002E-2</v>
       </c>
-      <c r="V125" s="2" t="s">
+      <c r="W125" s="2" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="126" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:23" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="4" t="s">
         <v>137</v>
       </c>
@@ -8789,10 +8926,10 @@
       <c r="D126" s="12" t="s">
         <v>298</v>
       </c>
-      <c r="E126" s="21" t="s">
+      <c r="E126" s="19" t="s">
         <v>654</v>
       </c>
-      <c r="F126" s="21" t="s">
+      <c r="F126" s="19" t="s">
         <v>654</v>
       </c>
       <c r="G126" s="12">
@@ -8808,18 +8945,19 @@
       </c>
       <c r="M126" s="14"/>
       <c r="O126" s="14"/>
-      <c r="Q126" s="4">
+      <c r="P126" s="14"/>
+      <c r="R126" s="4">
         <v>154</v>
       </c>
-      <c r="R126" s="4">
+      <c r="S126" s="4">
         <v>0.33600000000000002</v>
       </c>
-      <c r="S126" s="14"/>
-      <c r="V126" s="12" t="s">
+      <c r="T126" s="14"/>
+      <c r="W126" s="12" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="127" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:23" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="4" t="s">
         <v>138</v>
       </c>
@@ -8832,10 +8970,10 @@
       <c r="D127" s="12" t="s">
         <v>299</v>
       </c>
-      <c r="E127" s="21" t="s">
+      <c r="E127" s="19" t="s">
         <v>653</v>
       </c>
-      <c r="F127" s="21" t="s">
+      <c r="F127" s="19" t="s">
         <v>653</v>
       </c>
       <c r="G127" s="12">
@@ -8851,18 +8989,19 @@
       </c>
       <c r="M127" s="14"/>
       <c r="O127" s="14"/>
-      <c r="Q127" s="4">
+      <c r="P127" s="14"/>
+      <c r="R127" s="4">
         <v>103</v>
       </c>
-      <c r="R127" s="4">
+      <c r="S127" s="4">
         <v>0.224</v>
       </c>
-      <c r="S127" s="14"/>
-      <c r="V127" s="12" t="s">
+      <c r="T127" s="14"/>
+      <c r="W127" s="12" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="128" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>139</v>
       </c>
@@ -8889,17 +9028,17 @@
       <c r="L128">
         <v>0.48299999999999998</v>
       </c>
-      <c r="Q128">
+      <c r="R128">
         <v>241</v>
       </c>
-      <c r="R128">
+      <c r="S128">
         <v>0.52500000000000002</v>
       </c>
-      <c r="V128" s="2" t="s">
+      <c r="W128" s="2" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="129" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>140</v>
       </c>
@@ -8926,17 +9065,17 @@
       <c r="L129">
         <v>0.76100000000000001</v>
       </c>
-      <c r="Q129">
+      <c r="R129">
         <v>342</v>
       </c>
-      <c r="R129">
+      <c r="S129">
         <v>0.745</v>
       </c>
-      <c r="V129" s="2" t="s">
+      <c r="W129" s="2" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="130" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>141</v>
       </c>
@@ -8979,26 +9118,29 @@
       <c r="O130" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="P130" t="s">
+      <c r="P130" s="12" t="s">
+        <v>652</v>
+      </c>
+      <c r="Q130" t="s">
         <v>143</v>
       </c>
-      <c r="Q130">
+      <c r="R130">
         <v>5</v>
       </c>
-      <c r="R130">
+      <c r="S130">
         <v>1.0999999999999999E-2</v>
       </c>
-      <c r="S130" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="T130" t="s">
+      <c r="T130" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="U130" t="s">
         <v>143</v>
       </c>
-      <c r="V130" s="2" t="s">
+      <c r="W130" s="2" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="131" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>142</v>
       </c>
@@ -9036,20 +9178,20 @@
       <c r="O131" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q131">
+      <c r="R131">
         <v>153</v>
       </c>
-      <c r="R131">
+      <c r="S131">
         <v>0.33300000000000002</v>
       </c>
-      <c r="S131" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V131" s="2" t="s">
+      <c r="T131" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W131" s="2" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="132" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:23" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="4" t="s">
         <v>143</v>
       </c>
@@ -9090,20 +9232,21 @@
       <c r="O132" s="14" t="s">
         <v>325</v>
       </c>
-      <c r="Q132" s="4">
+      <c r="P132" s="14"/>
+      <c r="R132" s="4">
         <v>27</v>
       </c>
-      <c r="R132" s="4">
+      <c r="S132" s="4">
         <v>5.8999999999999997E-2</v>
       </c>
-      <c r="S132" s="14" t="s">
-        <v>325</v>
-      </c>
-      <c r="V132" s="12" t="s">
+      <c r="T132" s="14" t="s">
+        <v>325</v>
+      </c>
+      <c r="W132" s="12" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="133" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>144</v>
       </c>
@@ -9147,26 +9290,29 @@
       <c r="O133" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="P133" t="s">
+      <c r="P133" s="12" t="s">
+        <v>652</v>
+      </c>
+      <c r="Q133" t="s">
         <v>143</v>
       </c>
-      <c r="Q133">
+      <c r="R133">
         <v>3</v>
       </c>
-      <c r="R133">
+      <c r="S133">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="S133" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="T133" t="s">
+      <c r="T133" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="U133" t="s">
         <v>143</v>
       </c>
-      <c r="V133" s="2" t="s">
+      <c r="W133" s="2" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="134" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>145</v>
       </c>
@@ -9209,20 +9355,20 @@
       <c r="O134" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q134">
+      <c r="R134">
         <v>39</v>
       </c>
-      <c r="R134">
+      <c r="S134">
         <v>8.5000000000000006E-2</v>
       </c>
-      <c r="S134" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V134" s="2" t="s">
+      <c r="T134" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W134" s="2" t="s">
         <v>363</v>
       </c>
     </row>
-    <row r="135" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>146</v>
       </c>
@@ -9263,20 +9409,20 @@
       <c r="O135" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q135">
+      <c r="R135">
         <v>73</v>
       </c>
-      <c r="R135">
+      <c r="S135">
         <v>0.159</v>
       </c>
-      <c r="S135" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V135" s="2" t="s">
+      <c r="T135" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W135" s="2" t="s">
         <v>364</v>
       </c>
     </row>
-    <row r="136" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>147</v>
       </c>
@@ -9319,26 +9465,29 @@
       <c r="O136" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="P136" t="s">
+      <c r="P136" s="12" t="s">
+        <v>652</v>
+      </c>
+      <c r="Q136" t="s">
         <v>143</v>
       </c>
-      <c r="Q136">
+      <c r="R136">
         <v>4</v>
       </c>
-      <c r="R136">
+      <c r="S136">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="S136" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="T136" t="s">
+      <c r="T136" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="U136" t="s">
         <v>143</v>
       </c>
-      <c r="V136" s="2" t="s">
+      <c r="W136" s="2" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="137" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>148</v>
       </c>
@@ -9381,20 +9530,20 @@
       <c r="O137" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="Q137">
+      <c r="R137">
         <v>200</v>
       </c>
-      <c r="R137">
+      <c r="S137">
         <v>0.436</v>
       </c>
-      <c r="S137" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="V137" s="2" t="s">
+      <c r="T137" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="W137" s="2" t="s">
         <v>366</v>
       </c>
     </row>
-    <row r="138" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>149</v>
       </c>
@@ -9437,22 +9586,25 @@
       <c r="O138" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="P138" t="s">
+      <c r="P138" s="12" t="s">
+        <v>652</v>
+      </c>
+      <c r="Q138" t="s">
         <v>143</v>
       </c>
-      <c r="Q138">
+      <c r="R138">
         <v>4</v>
       </c>
-      <c r="R138">
+      <c r="S138">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="S138" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="T138" t="s">
+      <c r="T138" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="U138" t="s">
         <v>143</v>
       </c>
-      <c r="V138" s="2" t="s">
+      <c r="W138" s="2" t="s">
         <v>302</v>
       </c>
     </row>
@@ -9470,7 +9622,7 @@
       <formula>0.02</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R2:R138">
+  <conditionalFormatting sqref="S2:S138">
     <cfRule type="cellIs" dxfId="4" priority="7" operator="lessThan">
       <formula>0.02</formula>
     </cfRule>
@@ -9486,33 +9638,33 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:V76"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="73.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="73.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="83" customWidth="1"/>
-    <col min="6" max="6" width="79.44140625" customWidth="1"/>
-    <col min="7" max="7" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="79.42578125" customWidth="1"/>
+    <col min="7" max="7" width="7.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="14" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.5546875" style="5" customWidth="1"/>
-    <col min="14" max="14" width="23.77734375" customWidth="1"/>
-    <col min="15" max="15" width="8.33203125" style="5" customWidth="1"/>
-    <col min="16" max="16" width="37.21875" customWidth="1"/>
-    <col min="17" max="17" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.21875" style="5" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="29.88671875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="26.6640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="73.21875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5.5703125" style="5" customWidth="1"/>
+    <col min="14" max="14" width="23.7109375" customWidth="1"/>
+    <col min="15" max="15" width="8.28515625" style="5" customWidth="1"/>
+    <col min="16" max="16" width="37.28515625" customWidth="1"/>
+    <col min="17" max="17" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="29.85546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="73.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -9580,7 +9732,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>150</v>
       </c>
@@ -9622,7 +9774,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>151</v>
       </c>
@@ -9664,7 +9816,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>152</v>
       </c>
@@ -9706,7 +9858,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>153</v>
       </c>
@@ -9750,7 +9902,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>154</v>
       </c>
@@ -9795,7 +9947,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>155</v>
       </c>
@@ -9839,7 +9991,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>156</v>
       </c>
@@ -9883,7 +10035,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>157</v>
       </c>
@@ -9925,7 +10077,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>158</v>
       </c>
@@ -9969,7 +10121,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>159</v>
       </c>
@@ -10014,7 +10166,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>160</v>
       </c>
@@ -10059,7 +10211,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>161</v>
       </c>
@@ -10106,7 +10258,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>162</v>
       </c>
@@ -10157,7 +10309,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>163</v>
       </c>
@@ -10213,7 +10365,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>164</v>
       </c>
@@ -10258,7 +10410,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>165</v>
       </c>
@@ -10305,7 +10457,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>166</v>
       </c>
@@ -10352,7 +10504,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>167</v>
       </c>
@@ -10399,7 +10551,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>168</v>
       </c>
@@ -10446,7 +10598,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>169</v>
       </c>
@@ -10493,7 +10645,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>170</v>
       </c>
@@ -10540,7 +10692,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>171</v>
       </c>
@@ -10587,7 +10739,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>172</v>
       </c>
@@ -10632,7 +10784,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>173</v>
       </c>
@@ -10677,7 +10829,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>174</v>
       </c>
@@ -10724,7 +10876,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>175</v>
       </c>
@@ -10769,7 +10921,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>176</v>
       </c>
@@ -10816,7 +10968,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>177</v>
       </c>
@@ -10863,7 +11015,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>178</v>
       </c>
@@ -10910,7 +11062,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>179</v>
       </c>
@@ -10955,7 +11107,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>180</v>
       </c>
@@ -11002,7 +11154,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>181</v>
       </c>
@@ -11058,7 +11210,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>182</v>
       </c>
@@ -11105,7 +11257,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>183</v>
       </c>
@@ -11152,7 +11304,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>184</v>
       </c>
@@ -11197,7 +11349,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>185</v>
       </c>
@@ -11242,7 +11394,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>186</v>
       </c>
@@ -11289,7 +11441,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>187</v>
       </c>
@@ -11334,7 +11486,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>188</v>
       </c>
@@ -11379,7 +11531,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>70</v>
       </c>
@@ -11421,7 +11573,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>189</v>
       </c>
@@ -11463,7 +11615,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>71</v>
       </c>
@@ -11505,7 +11657,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>190</v>
       </c>
@@ -11553,7 +11705,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>191</v>
       </c>
@@ -11598,7 +11750,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>192</v>
       </c>
@@ -11643,7 +11795,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>193</v>
       </c>
@@ -11688,7 +11840,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>194</v>
       </c>
@@ -11733,7 +11885,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>195</v>
       </c>
@@ -11780,7 +11932,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>196</v>
       </c>
@@ -11836,7 +11988,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>197</v>
       </c>
@@ -11892,7 +12044,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>198</v>
       </c>
@@ -11937,7 +12089,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>199</v>
       </c>
@@ -11984,7 +12136,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>79</v>
       </c>
@@ -12021,7 +12173,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>200</v>
       </c>
@@ -12069,7 +12221,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>201</v>
       </c>
@@ -12117,7 +12269,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>202</v>
       </c>
@@ -12165,7 +12317,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>203</v>
       </c>
@@ -12213,7 +12365,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>204</v>
       </c>
@@ -12252,7 +12404,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>205</v>
       </c>
@@ -12300,7 +12452,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>206</v>
       </c>
@@ -12342,7 +12494,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>207</v>
       </c>
@@ -12395,7 +12547,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>100</v>
       </c>
@@ -12440,7 +12592,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>208</v>
       </c>
@@ -12482,7 +12634,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>209</v>
       </c>
@@ -12527,7 +12679,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>210</v>
       </c>
@@ -12572,7 +12724,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>211</v>
       </c>
@@ -12616,7 +12768,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="68" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:22" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
         <v>212</v>
       </c>
@@ -12664,7 +12816,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>213</v>
       </c>
@@ -12714,7 +12866,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>214</v>
       </c>
@@ -12758,7 +12910,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>215</v>
       </c>
@@ -12802,7 +12954,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>216</v>
       </c>
@@ -12847,7 +12999,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>217</v>
       </c>
@@ -12894,7 +13046,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="74" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>218</v>
       </c>
@@ -12941,7 +13093,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>219</v>
       </c>
@@ -12986,7 +13138,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>220</v>
       </c>

</xml_diff>